<commit_message>
feat: add scripts to consolidate and validate employee attendance data from XLSX files
</commit_message>
<xml_diff>
--- a/ملف حضور شهر 7/Combined_July.xlsx
+++ b/ملف حضور شهر 7/Combined_July.xlsx
@@ -445,7 +445,7 @@
         <v>حاضر</v>
       </c>
       <c r="G2" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -497,7 +497,7 @@
         <v>حاضر</v>
       </c>
       <c r="G4" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -523,7 +523,7 @@
         <v>حاضر</v>
       </c>
       <c r="G5" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -549,7 +549,7 @@
         <v>حاضر</v>
       </c>
       <c r="G6" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -575,7 +575,7 @@
         <v>حاضر</v>
       </c>
       <c r="G7" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -601,7 +601,7 @@
         <v>حاضر</v>
       </c>
       <c r="G8" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -627,7 +627,7 @@
         <v>حاضر</v>
       </c>
       <c r="G9" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -679,7 +679,7 @@
         <v>حاضر</v>
       </c>
       <c r="G11" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -705,7 +705,7 @@
         <v>حاضر</v>
       </c>
       <c r="G12" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -731,7 +731,7 @@
         <v>حاضر</v>
       </c>
       <c r="G13" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -757,7 +757,7 @@
         <v>حاضر</v>
       </c>
       <c r="G14" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>حاضر</v>
       </c>
       <c r="G15" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -809,7 +809,7 @@
         <v>حاضر</v>
       </c>
       <c r="G16" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -861,7 +861,7 @@
         <v>حاضر</v>
       </c>
       <c r="G18" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>حاضر</v>
       </c>
       <c r="G19" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -913,7 +913,7 @@
         <v>حاضر</v>
       </c>
       <c r="G20" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -939,7 +939,7 @@
         <v>حاضر</v>
       </c>
       <c r="G21" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -965,7 +965,7 @@
         <v>حاضر</v>
       </c>
       <c r="G22" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -991,7 +991,7 @@
         <v>حاضر</v>
       </c>
       <c r="G23" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1043,7 +1043,7 @@
         <v>حاضر</v>
       </c>
       <c r="G25" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1069,7 +1069,7 @@
         <v>حاضر</v>
       </c>
       <c r="G26" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1095,7 +1095,7 @@
         <v>حاضر</v>
       </c>
       <c r="G27" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -1121,7 +1121,7 @@
         <v>حاضر</v>
       </c>
       <c r="G28" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1147,7 +1147,7 @@
         <v>حاضر</v>
       </c>
       <c r="G29" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1173,7 +1173,7 @@
         <v>حاضر</v>
       </c>
       <c r="G30" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -1225,7 +1225,7 @@
         <v>حاضر</v>
       </c>
       <c r="G32" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -1251,7 +1251,7 @@
         <v>حاضر</v>
       </c>
       <c r="G33" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -1277,7 +1277,7 @@
         <v>حاضر</v>
       </c>
       <c r="G34" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -1303,7 +1303,7 @@
         <v>حاضر</v>
       </c>
       <c r="G35" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -1329,7 +1329,7 @@
         <v>حاضر</v>
       </c>
       <c r="G36" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -1355,7 +1355,7 @@
         <v>حاضر</v>
       </c>
       <c r="G37" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -1407,7 +1407,7 @@
         <v>حاضر</v>
       </c>
       <c r="G39" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -1433,7 +1433,7 @@
         <v>حاضر</v>
       </c>
       <c r="G40" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -1459,7 +1459,7 @@
         <v>حاضر</v>
       </c>
       <c r="G41" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -1485,7 +1485,7 @@
         <v>حاضر</v>
       </c>
       <c r="G42" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H42" t="str">
         <v/>
@@ -1511,7 +1511,7 @@
         <v>حاضر</v>
       </c>
       <c r="G43" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -1537,7 +1537,7 @@
         <v>حاضر</v>
       </c>
       <c r="G44" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -1589,7 +1589,7 @@
         <v>حاضر</v>
       </c>
       <c r="G46" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -1615,7 +1615,7 @@
         <v>حاضر</v>
       </c>
       <c r="G47" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -1641,7 +1641,7 @@
         <v>حاضر</v>
       </c>
       <c r="G48" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -1667,7 +1667,7 @@
         <v>حاضر</v>
       </c>
       <c r="G49" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -1693,7 +1693,7 @@
         <v>حاضر</v>
       </c>
       <c r="G50" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -1719,7 +1719,7 @@
         <v>حاضر</v>
       </c>
       <c r="G51" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H51" t="str">
         <v/>
@@ -1771,7 +1771,7 @@
         <v>حاضر</v>
       </c>
       <c r="G53" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H53" t="str">
         <v>4 ساعات اضافي حضور ليلا</v>
@@ -1797,7 +1797,7 @@
         <v>حاضر</v>
       </c>
       <c r="G54" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -1823,7 +1823,7 @@
         <v>حاضر</v>
       </c>
       <c r="G55" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -1849,7 +1849,7 @@
         <v>حاضر</v>
       </c>
       <c r="G56" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -1875,7 +1875,7 @@
         <v>حاضر</v>
       </c>
       <c r="G57" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -1901,7 +1901,7 @@
         <v>حاضر</v>
       </c>
       <c r="G58" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -1927,7 +1927,7 @@
         <v>حاضر</v>
       </c>
       <c r="G59" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -1979,7 +1979,7 @@
         <v>حاضر</v>
       </c>
       <c r="G61" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -2005,7 +2005,7 @@
         <v>حاضر</v>
       </c>
       <c r="G62" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -2031,7 +2031,7 @@
         <v>حاضر</v>
       </c>
       <c r="G63" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -2057,7 +2057,7 @@
         <v>حاضر</v>
       </c>
       <c r="G64" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -2109,7 +2109,7 @@
         <v>حاضر</v>
       </c>
       <c r="G66" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -2135,7 +2135,7 @@
         <v>حاضر</v>
       </c>
       <c r="G67" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -2161,7 +2161,7 @@
         <v>حاضر</v>
       </c>
       <c r="G68" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -2187,7 +2187,7 @@
         <v>حاضر</v>
       </c>
       <c r="G69" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -2213,7 +2213,7 @@
         <v>حاضر</v>
       </c>
       <c r="G70" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -2239,7 +2239,7 @@
         <v>حاضر</v>
       </c>
       <c r="G71" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H71" t="str">
         <v/>
@@ -2291,7 +2291,7 @@
         <v>حاضر</v>
       </c>
       <c r="G73" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H73" t="str">
         <v/>
@@ -2317,7 +2317,7 @@
         <v>حاضر</v>
       </c>
       <c r="G74" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H74" t="str">
         <v/>
@@ -2343,7 +2343,7 @@
         <v>حاضر</v>
       </c>
       <c r="G75" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H75" t="str">
         <v/>
@@ -2369,7 +2369,7 @@
         <v>حاضر</v>
       </c>
       <c r="G76" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H76" t="str">
         <v/>
@@ -2395,7 +2395,7 @@
         <v>حاضر</v>
       </c>
       <c r="G77" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H77" t="str">
         <v/>
@@ -2421,7 +2421,7 @@
         <v>حاضر</v>
       </c>
       <c r="G78" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -2447,7 +2447,7 @@
         <v>حاضر</v>
       </c>
       <c r="G79" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H79" t="str">
         <v/>
@@ -2473,7 +2473,7 @@
         <v>حاضر</v>
       </c>
       <c r="G80" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -2499,7 +2499,7 @@
         <v>حاضر</v>
       </c>
       <c r="G81" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -2525,7 +2525,7 @@
         <v>حاضر</v>
       </c>
       <c r="G82" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -2577,7 +2577,7 @@
         <v>حاضر</v>
       </c>
       <c r="G84" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -2603,7 +2603,7 @@
         <v>حاضر</v>
       </c>
       <c r="G85" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -2655,7 +2655,7 @@
         <v>حاضر</v>
       </c>
       <c r="G87" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -2681,7 +2681,7 @@
         <v>حاضر</v>
       </c>
       <c r="G88" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -2707,7 +2707,7 @@
         <v>حاضر</v>
       </c>
       <c r="G89" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -2733,7 +2733,7 @@
         <v>حاضر</v>
       </c>
       <c r="G90" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -2759,7 +2759,7 @@
         <v>حاضر</v>
       </c>
       <c r="G91" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -2785,7 +2785,7 @@
         <v>حاضر</v>
       </c>
       <c r="G92" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v>حاضر</v>
       </c>
       <c r="G94" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -2863,7 +2863,7 @@
         <v>حاضر</v>
       </c>
       <c r="G95" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -2889,7 +2889,7 @@
         <v>حاضر</v>
       </c>
       <c r="G96" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -2915,7 +2915,7 @@
         <v>غائب</v>
       </c>
       <c r="G97" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -2941,7 +2941,7 @@
         <v>غائب</v>
       </c>
       <c r="G98" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -2967,7 +2967,7 @@
         <v>غائب</v>
       </c>
       <c r="G99" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H99" t="str">
         <v/>
@@ -3019,7 +3019,7 @@
         <v>غائب</v>
       </c>
       <c r="G101" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -3045,7 +3045,7 @@
         <v>غائب</v>
       </c>
       <c r="G102" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H102" t="str">
         <v/>
@@ -3071,7 +3071,7 @@
         <v>غائب</v>
       </c>
       <c r="G103" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H103" t="str">
         <v/>
@@ -3097,7 +3097,7 @@
         <v>غائب</v>
       </c>
       <c r="G104" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H104" t="str">
         <v/>
@@ -3123,7 +3123,7 @@
         <v>غائب</v>
       </c>
       <c r="G105" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H105" t="str">
         <v/>
@@ -3149,7 +3149,7 @@
         <v>غائب</v>
       </c>
       <c r="G106" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H106" t="str">
         <v/>
@@ -3201,7 +3201,7 @@
         <v>غائب</v>
       </c>
       <c r="G108" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H108" t="str">
         <v/>
@@ -3227,7 +3227,7 @@
         <v>حاضر</v>
       </c>
       <c r="G109" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H109" t="str">
         <v/>
@@ -3253,7 +3253,7 @@
         <v>حاضر</v>
       </c>
       <c r="G110" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H110" t="str">
         <v/>
@@ -3279,7 +3279,7 @@
         <v>حاضر</v>
       </c>
       <c r="G111" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H111" t="str">
         <v/>
@@ -3305,7 +3305,7 @@
         <v>حاضر</v>
       </c>
       <c r="G112" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H112" t="str">
         <v/>
@@ -3331,7 +3331,7 @@
         <v>حاضر</v>
       </c>
       <c r="G113" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H113" t="str">
         <v/>
@@ -3383,7 +3383,7 @@
         <v>حاضر</v>
       </c>
       <c r="G115" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H115" t="str">
         <v/>
@@ -3409,7 +3409,7 @@
         <v>حاضر</v>
       </c>
       <c r="G116" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H116" t="str">
         <v/>
@@ -3435,7 +3435,7 @@
         <v>حاضر</v>
       </c>
       <c r="G117" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H117" t="str">
         <v/>
@@ -3461,7 +3461,7 @@
         <v>حاضر</v>
       </c>
       <c r="G118" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H118" t="str">
         <v/>
@@ -3487,7 +3487,7 @@
         <v>حاضر</v>
       </c>
       <c r="G119" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H119" t="str">
         <v/>
@@ -3513,7 +3513,7 @@
         <v>حاضر</v>
       </c>
       <c r="G120" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H120" t="str">
         <v/>
@@ -3539,7 +3539,7 @@
         <v>حاضر</v>
       </c>
       <c r="G121" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H121" t="str">
         <v/>
@@ -3547,7 +3547,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B122" t="str">
         <v>2026-07-01</v>
@@ -3565,7 +3565,7 @@
         <v>حاضر</v>
       </c>
       <c r="G122" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -3573,7 +3573,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B123" t="str">
         <v>2026-07-02</v>
@@ -3591,7 +3591,7 @@
         <v>حاضر</v>
       </c>
       <c r="G123" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H123" t="str">
         <v/>
@@ -3599,7 +3599,7 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B124" t="str">
         <v>2026-07-03</v>
@@ -3617,7 +3617,7 @@
         <v>حاضر</v>
       </c>
       <c r="G124" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -3625,7 +3625,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B125" t="str">
         <v>2026-07-04</v>
@@ -3651,7 +3651,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B126" t="str">
         <v>2026-07-05</v>
@@ -3669,7 +3669,7 @@
         <v>حاضر</v>
       </c>
       <c r="G126" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H126" t="str">
         <v/>
@@ -3677,7 +3677,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B127" t="str">
         <v>2026-07-06</v>
@@ -3695,7 +3695,7 @@
         <v>حاضر</v>
       </c>
       <c r="G127" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H127" t="str">
         <v/>
@@ -3703,7 +3703,7 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B128" t="str">
         <v>2026-07-07</v>
@@ -3721,7 +3721,7 @@
         <v>حاضر</v>
       </c>
       <c r="G128" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H128" t="str">
         <v/>
@@ -3729,7 +3729,7 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B129" t="str">
         <v>2026-07-08</v>
@@ -3747,7 +3747,7 @@
         <v>حاضر</v>
       </c>
       <c r="G129" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H129" t="str">
         <v/>
@@ -3755,7 +3755,7 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B130" t="str">
         <v>2026-07-09</v>
@@ -3773,7 +3773,7 @@
         <v>حاضر</v>
       </c>
       <c r="G130" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H130" t="str">
         <v/>
@@ -3781,7 +3781,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B131" t="str">
         <v>2026-07-10</v>
@@ -3799,7 +3799,7 @@
         <v>حاضر</v>
       </c>
       <c r="G131" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H131" t="str">
         <v/>
@@ -3807,7 +3807,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B132" t="str">
         <v>2026-07-11</v>
@@ -3825,7 +3825,7 @@
         <v>حاضر</v>
       </c>
       <c r="G132" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H132" t="str">
         <v/>
@@ -3833,7 +3833,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B133" t="str">
         <v>2026-07-12</v>
@@ -3851,7 +3851,7 @@
         <v>حاضر</v>
       </c>
       <c r="G133" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H133" t="str">
         <v/>
@@ -3859,7 +3859,7 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B134" t="str">
         <v>2026-07-13</v>
@@ -3877,7 +3877,7 @@
         <v>حاضر</v>
       </c>
       <c r="G134" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H134" t="str">
         <v/>
@@ -3885,7 +3885,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B135" t="str">
         <v>2026-07-14</v>
@@ -3903,7 +3903,7 @@
         <v>حاضر</v>
       </c>
       <c r="G135" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H135" t="str">
         <v/>
@@ -3911,7 +3911,7 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B136" t="str">
         <v>2026-07-15</v>
@@ -3929,7 +3929,7 @@
         <v>حاضر</v>
       </c>
       <c r="G136" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H136" t="str">
         <v/>
@@ -3937,7 +3937,7 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B137" t="str">
         <v>2026-07-16</v>
@@ -3955,7 +3955,7 @@
         <v>حاضر</v>
       </c>
       <c r="G137" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H137" t="str">
         <v/>
@@ -3963,7 +3963,7 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B138" t="str">
         <v>2026-07-17</v>
@@ -3981,7 +3981,7 @@
         <v>حاضر</v>
       </c>
       <c r="G138" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H138" t="str">
         <v/>
@@ -3989,7 +3989,7 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B139" t="str">
         <v>2026-07-18</v>
@@ -4015,7 +4015,7 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B140" t="str">
         <v>2026-07-19</v>
@@ -4041,7 +4041,7 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B141" t="str">
         <v>2026-07-20</v>
@@ -4059,7 +4059,7 @@
         <v>حاضر</v>
       </c>
       <c r="G141" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H141" t="str">
         <v/>
@@ -4067,7 +4067,7 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B142" t="str">
         <v>2026-07-21</v>
@@ -4085,7 +4085,7 @@
         <v>حاضر</v>
       </c>
       <c r="G142" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H142" t="str">
         <v/>
@@ -4093,7 +4093,7 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B143" t="str">
         <v>2026-07-22</v>
@@ -4111,7 +4111,7 @@
         <v>حاضر</v>
       </c>
       <c r="G143" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H143" t="str">
         <v/>
@@ -4119,7 +4119,7 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B144" t="str">
         <v>2026-07-23</v>
@@ -4137,7 +4137,7 @@
         <v>حاضر</v>
       </c>
       <c r="G144" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H144" t="str">
         <v/>
@@ -4145,7 +4145,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B145" t="str">
         <v>2026-07-24</v>
@@ -4163,7 +4163,7 @@
         <v>حاضر</v>
       </c>
       <c r="G145" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H145" t="str">
         <v/>
@@ -4171,7 +4171,7 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B146" t="str">
         <v>2026-07-25</v>
@@ -4197,7 +4197,7 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B147" t="str">
         <v>2026-07-26</v>
@@ -4215,7 +4215,7 @@
         <v>حاضر</v>
       </c>
       <c r="G147" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H147" t="str">
         <v/>
@@ -4223,7 +4223,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B148" t="str">
         <v>2026-07-27</v>
@@ -4241,7 +4241,7 @@
         <v>حاضر</v>
       </c>
       <c r="G148" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H148" t="str">
         <v/>
@@ -4249,7 +4249,7 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B149" t="str">
         <v>2026-07-28</v>
@@ -4267,7 +4267,7 @@
         <v>حاضر</v>
       </c>
       <c r="G149" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H149" t="str">
         <v/>
@@ -4275,7 +4275,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B150" t="str">
         <v>2026-07-29</v>
@@ -4293,7 +4293,7 @@
         <v>حاضر</v>
       </c>
       <c r="G150" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H150" t="str">
         <v/>
@@ -4301,7 +4301,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>بدر</v>
+        <v>بدر علاء</v>
       </c>
       <c r="B151" t="str">
         <v>2026-07-30</v>
@@ -4319,7 +4319,7 @@
         <v>حاضر</v>
       </c>
       <c r="G151" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H151" t="str">
         <v/>
@@ -4327,7 +4327,7 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B152" t="str">
         <v>2026-07-01</v>
@@ -4345,7 +4345,7 @@
         <v>حاضر</v>
       </c>
       <c r="G152" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H152" t="str">
         <v/>
@@ -4353,7 +4353,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B153" t="str">
         <v>2026-07-02</v>
@@ -4379,7 +4379,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B154" t="str">
         <v>2026-07-03</v>
@@ -4397,7 +4397,7 @@
         <v>حاضر</v>
       </c>
       <c r="G154" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H154" t="str">
         <v/>
@@ -4405,7 +4405,7 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B155" t="str">
         <v>2026-07-04</v>
@@ -4423,7 +4423,7 @@
         <v>حاضر</v>
       </c>
       <c r="G155" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H155" t="str">
         <v/>
@@ -4431,7 +4431,7 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B156" t="str">
         <v>2026-07-05</v>
@@ -4449,7 +4449,7 @@
         <v>حاضر</v>
       </c>
       <c r="G156" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H156" t="str">
         <v/>
@@ -4457,7 +4457,7 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B157" t="str">
         <v>2026-07-06</v>
@@ -4475,7 +4475,7 @@
         <v>حاضر</v>
       </c>
       <c r="G157" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H157" t="str">
         <v/>
@@ -4483,7 +4483,7 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B158" t="str">
         <v>2026-07-07</v>
@@ -4501,7 +4501,7 @@
         <v>حاضر</v>
       </c>
       <c r="G158" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H158" t="str">
         <v/>
@@ -4509,7 +4509,7 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B159" t="str">
         <v>2026-07-08</v>
@@ -4527,7 +4527,7 @@
         <v>حاضر</v>
       </c>
       <c r="G159" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H159" t="str">
         <v/>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B160" t="str">
         <v>2026-07-09</v>
@@ -4553,7 +4553,7 @@
         <v>حاضر</v>
       </c>
       <c r="G160" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H160" t="str">
         <v/>
@@ -4561,7 +4561,7 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B161" t="str">
         <v>2026-07-10</v>
@@ -4579,7 +4579,7 @@
         <v>حاضر</v>
       </c>
       <c r="G161" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H161" t="str">
         <v/>
@@ -4587,7 +4587,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B162" t="str">
         <v>2026-07-11</v>
@@ -4613,7 +4613,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B163" t="str">
         <v>2026-07-12</v>
@@ -4631,7 +4631,7 @@
         <v>حاضر</v>
       </c>
       <c r="G163" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H163" t="str">
         <v/>
@@ -4639,7 +4639,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B164" t="str">
         <v>2026-07-13</v>
@@ -4657,7 +4657,7 @@
         <v>حاضر</v>
       </c>
       <c r="G164" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H164" t="str">
         <v/>
@@ -4665,7 +4665,7 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B165" t="str">
         <v>2026-07-14</v>
@@ -4683,7 +4683,7 @@
         <v>حاضر</v>
       </c>
       <c r="G165" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H165" t="str">
         <v/>
@@ -4691,7 +4691,7 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B166" t="str">
         <v>2026-07-15</v>
@@ -4709,7 +4709,7 @@
         <v>حاضر</v>
       </c>
       <c r="G166" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H166" t="str">
         <v/>
@@ -4717,7 +4717,7 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B167" t="str">
         <v>2026-07-16</v>
@@ -4735,7 +4735,7 @@
         <v>حاضر</v>
       </c>
       <c r="G167" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H167" t="str">
         <v/>
@@ -4743,7 +4743,7 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B168" t="str">
         <v>2026-07-17</v>
@@ -4769,7 +4769,7 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B169" t="str">
         <v>2026-07-18</v>
@@ -4787,7 +4787,7 @@
         <v>حاضر</v>
       </c>
       <c r="G169" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H169" t="str">
         <v/>
@@ -4795,7 +4795,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B170" t="str">
         <v>2026-07-19</v>
@@ -4813,7 +4813,7 @@
         <v>حاضر</v>
       </c>
       <c r="G170" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H170" t="str">
         <v/>
@@ -4821,7 +4821,7 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B171" t="str">
         <v>2026-07-20</v>
@@ -4839,7 +4839,7 @@
         <v>حاضر</v>
       </c>
       <c r="G171" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H171" t="str">
         <v/>
@@ -4847,7 +4847,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B172" t="str">
         <v>2026-07-21</v>
@@ -4865,7 +4865,7 @@
         <v>حاضر</v>
       </c>
       <c r="G172" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H172" t="str">
         <v/>
@@ -4873,7 +4873,7 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B173" t="str">
         <v>2026-07-22</v>
@@ -4891,7 +4891,7 @@
         <v>حاضر</v>
       </c>
       <c r="G173" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H173" t="str">
         <v/>
@@ -4899,7 +4899,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B174" t="str">
         <v>2026-07-23</v>
@@ -4917,7 +4917,7 @@
         <v>حاضر</v>
       </c>
       <c r="G174" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H174" t="str">
         <v/>
@@ -4925,7 +4925,7 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B175" t="str">
         <v>2026-07-24</v>
@@ -4943,7 +4943,7 @@
         <v>حاضر</v>
       </c>
       <c r="G175" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H175" t="str">
         <v/>
@@ -4951,7 +4951,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B176" t="str">
         <v>2026-07-25</v>
@@ -4977,7 +4977,7 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B177" t="str">
         <v>2026-07-26</v>
@@ -4995,7 +4995,7 @@
         <v>حاضر</v>
       </c>
       <c r="G177" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H177" t="str">
         <v/>
@@ -5003,7 +5003,7 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B178" t="str">
         <v>2026-07-27</v>
@@ -5021,7 +5021,7 @@
         <v>حاضر</v>
       </c>
       <c r="G178" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H178" t="str">
         <v/>
@@ -5029,7 +5029,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B179" t="str">
         <v>2026-07-28</v>
@@ -5047,7 +5047,7 @@
         <v>حاضر</v>
       </c>
       <c r="G179" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H179" t="str">
         <v/>
@@ -5055,7 +5055,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B180" t="str">
         <v>2026-07-29</v>
@@ -5073,7 +5073,7 @@
         <v>حاضر</v>
       </c>
       <c r="G180" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H180" t="str">
         <v/>
@@ -5081,7 +5081,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>اموله</v>
+        <v>امل</v>
       </c>
       <c r="B181" t="str">
         <v>2026-07-30</v>
@@ -5099,7 +5099,7 @@
         <v>حاضر</v>
       </c>
       <c r="G181" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H181" t="str">
         <v/>
@@ -5125,7 +5125,7 @@
         <v>حاضر</v>
       </c>
       <c r="G182" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H182" t="str">
         <v/>
@@ -5151,7 +5151,7 @@
         <v>حاضر</v>
       </c>
       <c r="G183" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H183" t="str">
         <v/>
@@ -5177,7 +5177,7 @@
         <v>حاضر</v>
       </c>
       <c r="G184" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H184" t="str">
         <v/>
@@ -5229,7 +5229,7 @@
         <v>حاضر</v>
       </c>
       <c r="G186" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H186" t="str">
         <v/>
@@ -5255,7 +5255,7 @@
         <v>حاضر</v>
       </c>
       <c r="G187" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H187" t="str">
         <v/>
@@ -5281,7 +5281,7 @@
         <v>حاضر</v>
       </c>
       <c r="G188" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H188" t="str">
         <v/>
@@ -5307,7 +5307,7 @@
         <v>حاضر</v>
       </c>
       <c r="G189" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H189" t="str">
         <v/>
@@ -5359,7 +5359,7 @@
         <v>حاضر</v>
       </c>
       <c r="G191" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H191" t="str">
         <v/>
@@ -5385,7 +5385,7 @@
         <v>حاضر</v>
       </c>
       <c r="G192" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H192" t="str">
         <v/>
@@ -5411,7 +5411,7 @@
         <v>حاضر</v>
       </c>
       <c r="G193" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H193" t="str">
         <v/>
@@ -5437,7 +5437,7 @@
         <v>حاضر</v>
       </c>
       <c r="G194" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H194" t="str">
         <v/>
@@ -5463,7 +5463,7 @@
         <v>حاضر</v>
       </c>
       <c r="G195" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H195" t="str">
         <v/>
@@ -5489,7 +5489,7 @@
         <v>حاضر</v>
       </c>
       <c r="G196" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H196" t="str">
         <v/>
@@ -5515,7 +5515,7 @@
         <v>حاضر</v>
       </c>
       <c r="G197" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H197" t="str">
         <v/>
@@ -5541,7 +5541,7 @@
         <v>حاضر</v>
       </c>
       <c r="G198" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H198" t="str">
         <v/>
@@ -5567,7 +5567,7 @@
         <v>حاضر</v>
       </c>
       <c r="G199" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H199" t="str">
         <v/>
@@ -5593,7 +5593,7 @@
         <v>حاضر</v>
       </c>
       <c r="G200" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H200" t="str">
         <v/>
@@ -5619,7 +5619,7 @@
         <v>حاضر</v>
       </c>
       <c r="G201" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H201" t="str">
         <v/>
@@ -5645,7 +5645,7 @@
         <v>حاضر</v>
       </c>
       <c r="G202" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H202" t="str">
         <v/>
@@ -5671,7 +5671,7 @@
         <v>حاضر</v>
       </c>
       <c r="G203" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H203" t="str">
         <v/>
@@ -5723,7 +5723,7 @@
         <v>حاضر</v>
       </c>
       <c r="G205" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H205" t="str">
         <v/>
@@ -5749,7 +5749,7 @@
         <v>حاضر</v>
       </c>
       <c r="G206" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H206" t="str">
         <v/>
@@ -5775,7 +5775,7 @@
         <v>حاضر</v>
       </c>
       <c r="G207" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H207" t="str">
         <v/>
@@ -5801,7 +5801,7 @@
         <v>حاضر</v>
       </c>
       <c r="G208" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H208" t="str">
         <v/>
@@ -5827,7 +5827,7 @@
         <v>حاضر</v>
       </c>
       <c r="G209" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H209" t="str">
         <v/>
@@ -5853,7 +5853,7 @@
         <v>حاضر</v>
       </c>
       <c r="G210" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H210" t="str">
         <v/>
@@ -5905,7 +5905,7 @@
         <v>حاضر</v>
       </c>
       <c r="G212" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H212" t="str">
         <v/>
@@ -5931,7 +5931,7 @@
         <v>حاضر</v>
       </c>
       <c r="G213" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H213" t="str">
         <v/>
@@ -5983,7 +5983,7 @@
         <v>حاضر</v>
       </c>
       <c r="G215" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H215" t="str">
         <v/>
@@ -6009,7 +6009,7 @@
         <v>حاضر</v>
       </c>
       <c r="G216" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H216" t="str">
         <v/>
@@ -6035,7 +6035,7 @@
         <v>حاضر</v>
       </c>
       <c r="G217" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H217" t="str">
         <v/>
@@ -6061,7 +6061,7 @@
         <v>حاضر</v>
       </c>
       <c r="G218" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H218" t="str">
         <v/>
@@ -6087,7 +6087,7 @@
         <v>حاضر</v>
       </c>
       <c r="G219" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H219" t="str">
         <v/>
@@ -6113,7 +6113,7 @@
         <v>حاضر</v>
       </c>
       <c r="G220" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H220" t="str">
         <v/>
@@ -6165,7 +6165,7 @@
         <v>حاضر</v>
       </c>
       <c r="G222" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H222" t="str">
         <v/>
@@ -6191,7 +6191,7 @@
         <v>حاضر</v>
       </c>
       <c r="G223" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H223" t="str">
         <v/>
@@ -6217,7 +6217,7 @@
         <v>حاضر</v>
       </c>
       <c r="G224" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H224" t="str">
         <v/>
@@ -6243,7 +6243,7 @@
         <v>حاضر</v>
       </c>
       <c r="G225" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H225" t="str">
         <v/>
@@ -6269,7 +6269,7 @@
         <v>حاضر</v>
       </c>
       <c r="G226" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H226" t="str">
         <v/>
@@ -6295,7 +6295,7 @@
         <v>حاضر</v>
       </c>
       <c r="G227" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H227" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>حاضر</v>
       </c>
       <c r="G228" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H228" t="str">
         <v/>
@@ -6373,7 +6373,7 @@
         <v>حاضر</v>
       </c>
       <c r="G230" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H230" t="str">
         <v/>
@@ -6399,7 +6399,7 @@
         <v>حاضر</v>
       </c>
       <c r="G231" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H231" t="str">
         <v/>
@@ -6425,7 +6425,7 @@
         <v>حاضر</v>
       </c>
       <c r="G232" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H232" t="str">
         <v/>
@@ -6451,7 +6451,7 @@
         <v>حاضر</v>
       </c>
       <c r="G233" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H233" t="str">
         <v/>
@@ -6477,7 +6477,7 @@
         <v>حاضر</v>
       </c>
       <c r="G234" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H234" t="str">
         <v/>
@@ -6529,7 +6529,7 @@
         <v>حاضر</v>
       </c>
       <c r="G236" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H236" t="str">
         <v/>
@@ -6555,7 +6555,7 @@
         <v>حاضر</v>
       </c>
       <c r="G237" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H237" t="str">
         <v/>
@@ -6581,7 +6581,7 @@
         <v>حاضر</v>
       </c>
       <c r="G238" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H238" t="str">
         <v/>
@@ -6607,7 +6607,7 @@
         <v>حاضر</v>
       </c>
       <c r="G239" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H239" t="str">
         <v/>
@@ -6633,7 +6633,7 @@
         <v>حاضر</v>
       </c>
       <c r="G240" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H240" t="str">
         <v/>
@@ -6659,7 +6659,7 @@
         <v>حاضر</v>
       </c>
       <c r="G241" t="str">
-        <v>✅ تمت الموافقة</v>
+        <v/>
       </c>
       <c r="H241" t="str">
         <v/>

</xml_diff>